<commit_message>
branch for iicl backend with image upload and mail service
</commit_message>
<xml_diff>
--- a/docs/INCHCAPE PRICE LIST.xlsx
+++ b/docs/INCHCAPE PRICE LIST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Monthly Accounts\metals workshop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\damage-report\apps\web\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9238752A-04D5-42EC-B216-52BA3B6E8973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E183309-EEAD-48AB-9591-1AE0DF2FABC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{A452D54E-E95C-483D-8540-5BF96D640265}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A452D54E-E95C-483D-8540-5BF96D640265}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -775,9 +775,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -829,6 +826,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -847,9 +847,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -887,7 +887,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -993,7 +993,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1135,7 +1135,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1144,21 +1144,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C378CE5-CEAC-4435-A417-F6BBF7D35549}">
   <dimension ref="A1:G124"/>
-  <sheetFormatPr defaultColWidth="24.89453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="24.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.7890625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5234375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="55" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1015625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7890625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.89453125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="3" customWidth="1"/>
     <col min="7" max="7" width="65" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.1015625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.3125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="24.89453125" style="3"/>
+    <col min="8" max="8" width="13.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="24.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1174,12 +1174,12 @@
       <c r="E1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="G1" s="9"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G1" s="26"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1402,7 +1402,7 @@
       <c r="F12" s="7"/>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>1</v>
       </c>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>2</v>
       </c>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>3</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>4</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1491,7 +1491,7 @@
       <c r="F17" s="7"/>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>14</v>
       </c>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>15</v>
       </c>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>16</v>
       </c>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>17</v>
       </c>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>18</v>
       </c>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>19</v>
       </c>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1614,7 +1614,7 @@
       <c r="F24" s="7"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>20</v>
       </c>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G25" s="4"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="G26" s="4"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>22</v>
       </c>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>24</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1722,7 +1722,7 @@
       <c r="F30" s="7"/>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>25</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>26</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>27</v>
       </c>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>28</v>
       </c>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G34" s="4"/>
     </row>
-    <row r="35" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -1811,7 +1811,7 @@
       <c r="F35" s="7"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>30</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
         <v>31</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>32</v>
       </c>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="G38" s="4"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>33</v>
       </c>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G39" s="4"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>34</v>
       </c>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="G40" s="4"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>35</v>
       </c>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="G41" s="4"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>36</v>
       </c>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="G42" s="4"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>37</v>
       </c>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="G43" s="4"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>38</v>
       </c>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G44" s="4"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>39</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" s="4" t="s">
         <v>35</v>
@@ -2030,7 +2030,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>40</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -2062,7 +2062,7 @@
       <c r="F48" s="7"/>
       <c r="G48" s="6"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
         <v>41</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>42</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
         <v>43</v>
       </c>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
         <v>44</v>
       </c>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="G52" s="4"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
         <v>45</v>
       </c>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
         <v>46</v>
       </c>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
         <v>47</v>
       </c>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
         <v>48</v>
       </c>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
         <v>49</v>
       </c>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
         <v>50</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" s="4" t="s">
         <v>49</v>
@@ -2281,7 +2281,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="15.45" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:7" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
         <v>51</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -2313,7 +2313,7 @@
       <c r="F61" s="7"/>
       <c r="G61" s="6"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
         <v>52</v>
       </c>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="G62" s="4"/>
     </row>
-    <row r="63" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -2341,7 +2341,7 @@
       <c r="F63" s="7"/>
       <c r="G63" s="6"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
         <v>53</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
         <v>54</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
         <v>55</v>
       </c>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="G66" s="4"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
         <v>56</v>
       </c>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="G67" s="4"/>
     </row>
-    <row r="68" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="6"/>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -2430,7 +2430,7 @@
       <c r="F68" s="7"/>
       <c r="G68" s="6"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
         <v>57</v>
       </c>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
         <v>59</v>
       </c>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="G70" s="4"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
         <v>61</v>
       </c>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="6"/>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -2496,7 +2496,7 @@
       <c r="F72" s="7"/>
       <c r="G72" s="6"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
         <v>62</v>
       </c>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="G73" s="4"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
         <v>63</v>
       </c>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="G74" s="4"/>
     </row>
-    <row r="75" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -2543,7 +2543,7 @@
       <c r="F75" s="7"/>
       <c r="G75" s="6"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
         <v>64</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
         <v>65</v>
       </c>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="G77" s="4"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
         <v>66</v>
       </c>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="G78" s="4"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>67</v>
       </c>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="G79" s="4"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
         <v>68</v>
       </c>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="G80" s="4"/>
     </row>
-    <row r="81" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="6"/>
       <c r="B81" s="6"/>
       <c r="C81" s="6"/>
@@ -2649,7 +2649,7 @@
       <c r="F81" s="7"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
         <v>69</v>
       </c>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="G82" s="4"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="4">
         <v>70</v>
       </c>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="G83" s="4"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="4">
         <v>71</v>
       </c>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="G84" s="4"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="4">
         <v>72</v>
       </c>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="G85" s="4"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
         <v>73</v>
       </c>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="G86" s="4"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>74</v>
       </c>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="G87" s="4"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
         <v>75</v>
       </c>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="G88" s="4"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="4">
         <v>76</v>
       </c>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="G89" s="4"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="4">
         <v>77</v>
       </c>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="G90" s="4"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="4">
         <v>78</v>
       </c>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="G91" s="4"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
         <v>79</v>
       </c>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="G92" s="4"/>
     </row>
-    <row r="93" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
       <c r="B93" s="6"/>
       <c r="C93" s="6"/>
@@ -2867,7 +2867,7 @@
       <c r="F93" s="7"/>
       <c r="G93" s="6"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
         <v>80</v>
       </c>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="G94" s="4"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="4">
         <v>81</v>
       </c>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G95" s="4"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="4">
         <v>82</v>
       </c>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="G96" s="4"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="4">
         <v>83</v>
       </c>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="G97" s="4"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="4">
         <v>84</v>
       </c>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="G98" s="4"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="4">
         <v>85</v>
       </c>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="G99" s="4"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="4">
         <v>86</v>
       </c>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="G100" s="4"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="4">
         <v>87</v>
       </c>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="G101" s="4"/>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="4">
         <v>88</v>
       </c>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="G102" s="4"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
         <v>89</v>
       </c>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="G103" s="4"/>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="4">
         <v>90</v>
       </c>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="G104" s="4"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
         <v>91</v>
       </c>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="G105" s="4"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="4">
         <v>92</v>
       </c>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="G106" s="4"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="4">
         <v>93</v>
       </c>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="G107" s="4"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="4">
         <v>95</v>
       </c>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="G108" s="4"/>
     </row>
-    <row r="109" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A109" s="6"/>
       <c r="B109" s="6"/>
       <c r="C109" s="6"/>
@@ -3167,7 +3167,7 @@
       <c r="F109" s="7"/>
       <c r="G109" s="6"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="4">
         <v>96</v>
       </c>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="G110" s="4"/>
     </row>
-    <row r="111" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="111" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A111" s="6"/>
       <c r="B111" s="6"/>
       <c r="C111" s="6"/>
@@ -3195,7 +3195,7 @@
       <c r="F111" s="7"/>
       <c r="G111" s="6"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" s="4">
         <v>97</v>
       </c>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G112" s="4"/>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>98</v>
       </c>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="G113" s="4"/>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114" s="4">
         <v>99</v>
       </c>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="G114" s="4"/>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115" s="4">
         <v>100</v>
       </c>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="G115" s="4"/>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116" s="4">
         <v>101</v>
       </c>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="G116" s="4"/>
     </row>
-    <row r="117" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="117" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A117" s="6"/>
       <c r="B117" s="6"/>
       <c r="C117" s="6"/>
@@ -3305,7 +3305,7 @@
       <c r="F117" s="7"/>
       <c r="G117" s="6"/>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -3314,7 +3314,7 @@
       <c r="F118" s="4"/>
       <c r="G118" s="4"/>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -3323,7 +3323,7 @@
       <c r="F119" s="4"/>
       <c r="G119" s="4"/>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -3332,7 +3332,7 @@
       <c r="F120" s="4"/>
       <c r="G120" s="4"/>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
@@ -3341,7 +3341,7 @@
       <c r="F121" s="4"/>
       <c r="G121" s="4"/>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
@@ -3350,7 +3350,7 @@
       <c r="F122" s="4"/>
       <c r="G122" s="4"/>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
@@ -3359,7 +3359,7 @@
       <c r="F123" s="4"/>
       <c r="G123" s="4"/>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
@@ -3380,1016 +3380,1016 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A485C0-60AA-4FC3-B072-498078964BD7}">
   <dimension ref="A1:E78"/>
-  <sheetFormatPr defaultColWidth="24.89453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultColWidth="24.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.68359375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1015625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="55" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1015625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7890625" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="24.89453125" style="10"/>
+    <col min="4" max="4" width="14.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="24.88671875" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="35.700000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:5" ht="35.700000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="26"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="13" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="25"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="15" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="17">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="16">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>12000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="17">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="16">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="18">
+      <c r="D4" s="10"/>
+      <c r="E4" s="17">
         <v>3500</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="17">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="16">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="18">
+      <c r="D5" s="10"/>
+      <c r="E5" s="17">
         <v>3000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="17">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="16">
         <v>4</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="18">
+      <c r="D6" s="10"/>
+      <c r="E6" s="17">
         <v>2500</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="17">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="16">
         <v>5</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="18">
+      <c r="D7" s="10"/>
+      <c r="E7" s="17">
         <v>1500</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="17">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="16">
         <v>6</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <v>8000</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="19"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="20"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="17">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="18"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="19"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="16">
         <v>7</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="18">
+      <c r="D10" s="10"/>
+      <c r="E10" s="17">
         <v>800</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="17">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="16">
         <v>8</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="18">
+      <c r="D11" s="10"/>
+      <c r="E11" s="17">
         <v>1000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="19"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="20"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="17">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="18"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="19"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="16">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="18">
+      <c r="D13" s="10"/>
+      <c r="E13" s="17">
         <v>9000</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="17">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="16">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="18">
+      <c r="D14" s="10"/>
+      <c r="E14" s="17">
         <v>9000</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="17">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="16">
         <v>11</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="18">
+      <c r="D15" s="10"/>
+      <c r="E15" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="17">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="16">
         <v>12</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="18">
+      <c r="D16" s="10"/>
+      <c r="E16" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="19"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="20"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="18"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="19"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="16">
         <v>13</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="18">
+      <c r="D18" s="10"/>
+      <c r="E18" s="17">
         <v>12000</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="17">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="16">
         <v>14</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="18">
+      <c r="D19" s="10"/>
+      <c r="E19" s="17">
         <v>6000</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="17">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="16">
         <v>15</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="18">
+      <c r="D20" s="10"/>
+      <c r="E20" s="17">
         <v>4500</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="17">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="16">
         <v>16</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="18">
+      <c r="D21" s="10"/>
+      <c r="E21" s="17">
         <v>4500</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="19"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="20"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="17">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="18"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="19"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="16">
         <v>17</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="18">
+      <c r="D23" s="10"/>
+      <c r="E23" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="17">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="16">
         <v>18</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="18">
+      <c r="D24" s="10"/>
+      <c r="E24" s="17">
         <v>4500</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="17">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="16">
         <v>19</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="18">
+      <c r="D25" s="10"/>
+      <c r="E25" s="17">
         <v>3000</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="17">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="16">
         <v>20</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="18">
+      <c r="D26" s="10"/>
+      <c r="E26" s="17">
         <v>2000</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="19"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="20"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="17">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="18"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="19"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="16">
         <v>21</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="18">
+      <c r="D28" s="10"/>
+      <c r="E28" s="17">
         <v>12000</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="17">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="16">
         <v>22</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="18">
+      <c r="D29" s="10"/>
+      <c r="E29" s="17">
         <v>6000</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="17">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="16">
         <v>23</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="18">
+      <c r="D30" s="10"/>
+      <c r="E30" s="17">
         <v>1000</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="17">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="16">
         <v>24</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D31" s="11"/>
-      <c r="E31" s="18">
+      <c r="D31" s="10"/>
+      <c r="E31" s="17">
         <v>500</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="17">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="16">
         <v>25</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E32" s="18">
+      <c r="E32" s="17">
         <v>3500</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="19"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="20"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="17">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="18"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="19"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="16">
         <v>26</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D34" s="11"/>
-      <c r="E34" s="18">
+      <c r="D34" s="10"/>
+      <c r="E34" s="17">
         <v>12000</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="17">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="16">
         <v>27</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="11"/>
-      <c r="E35" s="18">
+      <c r="D35" s="10"/>
+      <c r="E35" s="17">
         <v>6000</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="17">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="16">
         <v>28</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="11"/>
-      <c r="E36" s="18">
+      <c r="D36" s="10"/>
+      <c r="E36" s="17">
         <v>4000</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="17">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="16">
         <v>29</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="18">
+      <c r="E37" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="17">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="16">
         <v>30</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="D38" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="18">
+      <c r="E38" s="17">
         <v>3000</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="19"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="20"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="17">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="18"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="19"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="16">
         <v>31</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D40" s="11"/>
-      <c r="E40" s="18">
+      <c r="D40" s="10"/>
+      <c r="E40" s="17">
         <v>9000</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="19"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="20"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="17">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="18"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="19"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="16">
         <v>32</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="11"/>
-      <c r="E42" s="18">
+      <c r="D42" s="10"/>
+      <c r="E42" s="17">
         <v>15000</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="17">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="16">
         <v>33</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="11"/>
-      <c r="E43" s="18">
+      <c r="D43" s="10"/>
+      <c r="E43" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="17">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="16">
         <v>34</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D44" s="11"/>
-      <c r="E44" s="18">
+      <c r="D44" s="10"/>
+      <c r="E44" s="17">
         <v>2500</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="17">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="16">
         <v>35</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D45" s="11"/>
-      <c r="E45" s="18">
+      <c r="D45" s="10"/>
+      <c r="E45" s="17">
         <v>6000</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="19"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="20"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="17">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="18"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="19"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="16">
         <v>36</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="D47" s="11"/>
-      <c r="E47" s="18">
+      <c r="D47" s="10"/>
+      <c r="E47" s="17">
         <v>1200</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="17">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="16">
         <v>37</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D48" s="11"/>
-      <c r="E48" s="18">
+      <c r="D48" s="10"/>
+      <c r="E48" s="17">
         <v>600</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="19"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="20"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" s="17">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="18"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="19"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="16">
         <v>38</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D50" s="11"/>
-      <c r="E50" s="18">
+      <c r="D50" s="10"/>
+      <c r="E50" s="17">
         <v>2500</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" s="17">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="16">
         <v>39</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D51" s="11"/>
-      <c r="E51" s="18">
+      <c r="D51" s="10"/>
+      <c r="E51" s="17">
         <v>2000</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A52" s="19"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="20"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A53" s="17">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="18"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="19"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="16">
         <v>40</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="B53" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D53" s="11"/>
-      <c r="E53" s="18">
+      <c r="D53" s="10"/>
+      <c r="E53" s="17">
         <v>9000</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="17">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="16">
         <v>41</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D54" s="11"/>
-      <c r="E54" s="18">
+      <c r="D54" s="10"/>
+      <c r="E54" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="17">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="16">
         <v>42</v>
       </c>
-      <c r="B55" s="11" t="s">
+      <c r="B55" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D55" s="11"/>
-      <c r="E55" s="18">
+      <c r="D55" s="10"/>
+      <c r="E55" s="17">
         <v>9000</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="17">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="16">
         <v>43</v>
       </c>
-      <c r="B56" s="11" t="s">
+      <c r="B56" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D56" s="11"/>
-      <c r="E56" s="18">
+      <c r="D56" s="10"/>
+      <c r="E56" s="17">
         <v>3000</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="19"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="20"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A58" s="17">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="18"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="19"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A58" s="16">
         <v>44</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D58" s="11"/>
-      <c r="E58" s="18">
+      <c r="D58" s="10"/>
+      <c r="E58" s="17">
         <v>2000</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="17">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="16">
         <v>45</v>
       </c>
-      <c r="B59" s="11" t="s">
+      <c r="B59" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="D59" s="11"/>
-      <c r="E59" s="18">
+      <c r="D59" s="10"/>
+      <c r="E59" s="17">
         <v>800</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="17">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" s="16">
         <v>46</v>
       </c>
-      <c r="B60" s="11" t="s">
+      <c r="B60" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D60" s="11"/>
-      <c r="E60" s="18">
+      <c r="D60" s="10"/>
+      <c r="E60" s="17">
         <v>650</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="17">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="16">
         <v>47</v>
       </c>
-      <c r="B61" s="11" t="s">
+      <c r="B61" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D61" s="11"/>
-      <c r="E61" s="18">
+      <c r="D61" s="10"/>
+      <c r="E61" s="17">
         <v>3000</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="17">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" s="16">
         <v>48</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D62" s="11" t="s">
+      <c r="D62" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E62" s="18">
+      <c r="E62" s="17">
         <v>2500</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="17">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" s="16">
         <v>49</v>
       </c>
-      <c r="B63" s="11" t="s">
+      <c r="B63" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C63" s="11" t="s">
+      <c r="C63" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D63" s="11"/>
-      <c r="E63" s="18">
+      <c r="D63" s="10"/>
+      <c r="E63" s="17">
         <v>1000</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="19"/>
-      <c r="B64" s="12"/>
-      <c r="C64" s="12"/>
-      <c r="D64" s="12"/>
-      <c r="E64" s="20"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="17">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" s="18"/>
+      <c r="B64" s="11"/>
+      <c r="C64" s="11"/>
+      <c r="D64" s="11"/>
+      <c r="E64" s="19"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" s="16">
         <v>50</v>
       </c>
-      <c r="B65" s="11" t="s">
+      <c r="B65" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="C65" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="D65" s="11"/>
-      <c r="E65" s="18">
+      <c r="D65" s="10"/>
+      <c r="E65" s="17">
         <v>2000</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A66" s="19"/>
-      <c r="B66" s="12"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="20"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="17">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" s="18"/>
+      <c r="B66" s="11"/>
+      <c r="C66" s="11"/>
+      <c r="D66" s="11"/>
+      <c r="E66" s="19"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" s="16">
         <v>51</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C67" s="11" t="s">
+      <c r="C67" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D67" s="11"/>
-      <c r="E67" s="18">
+      <c r="D67" s="10"/>
+      <c r="E67" s="17">
         <v>7000</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A68" s="17">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" s="16">
         <v>52</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="11"/>
-      <c r="E68" s="18">
+      <c r="D68" s="10"/>
+      <c r="E68" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="17">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" s="16">
         <v>53</v>
       </c>
-      <c r="B69" s="11" t="s">
+      <c r="B69" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C69" s="11" t="s">
+      <c r="C69" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D69" s="11" t="s">
+      <c r="D69" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="E69" s="18">
+      <c r="E69" s="17">
         <v>7000</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A70" s="17">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" s="16">
         <v>54</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="B70" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D70" s="11" t="s">
+      <c r="D70" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="E70" s="18">
+      <c r="E70" s="17">
         <v>5000</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A71" s="21"/>
-      <c r="B71" s="22"/>
-      <c r="C71" s="22"/>
-      <c r="D71" s="22"/>
-      <c r="E71" s="23"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="20"/>
+      <c r="B71" s="21"/>
+      <c r="C71" s="21"/>
+      <c r="D71" s="21"/>
+      <c r="E71" s="22"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>

</xml_diff>